<commit_message>
Update files for aggrecan and fold change in optimization workflow
</commit_message>
<xml_diff>
--- a/parameters.xlsx
+++ b/parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmunip.CAMPUS\source\repos\ABM-NM-optimization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1866BF85-0F64-4A90-AEE6-FC5B8EEDFB6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBBB0915-F895-47A8-B3CA-B325DDD7F822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14303" yWindow="-98" windowWidth="28995" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5670" yWindow="3720" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="81">
   <si>
     <t>Mean</t>
   </si>
@@ -731,6 +731,9 @@
       <c r="G3">
         <v>1</v>
       </c>
+      <c r="H3" t="s">
+        <v>10</v>
+      </c>
       <c r="J3">
         <v>1</v>
       </c>
@@ -761,6 +764,9 @@
       <c r="G4">
         <v>1</v>
       </c>
+      <c r="H4" t="s">
+        <v>10</v>
+      </c>
       <c r="J4">
         <v>2</v>
       </c>
@@ -791,6 +797,9 @@
       <c r="G5">
         <v>3</v>
       </c>
+      <c r="H5" t="s">
+        <v>10</v>
+      </c>
       <c r="J5">
         <v>3</v>
       </c>
@@ -821,6 +830,9 @@
       <c r="G6">
         <v>1</v>
       </c>
+      <c r="H6" t="s">
+        <v>10</v>
+      </c>
       <c r="J6">
         <v>4</v>
       </c>
@@ -851,6 +863,9 @@
       <c r="G7">
         <v>1</v>
       </c>
+      <c r="H7" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -875,6 +890,9 @@
       <c r="G8">
         <v>1</v>
       </c>
+      <c r="H8" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -899,6 +917,9 @@
       <c r="G9">
         <v>1</v>
       </c>
+      <c r="H9" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -923,6 +944,9 @@
       <c r="G10">
         <v>1</v>
       </c>
+      <c r="H10" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -946,6 +970,9 @@
       </c>
       <c r="G11">
         <v>1</v>
+      </c>
+      <c r="H11" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -971,6 +998,9 @@
       <c r="G12">
         <v>1</v>
       </c>
+      <c r="H12" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -995,6 +1025,9 @@
       <c r="G13">
         <v>1</v>
       </c>
+      <c r="H13" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -1019,6 +1052,9 @@
       <c r="G14">
         <v>1</v>
       </c>
+      <c r="H14" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -1043,6 +1079,9 @@
       <c r="G15">
         <v>1</v>
       </c>
+      <c r="H15" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -1235,20 +1274,23 @@
         <v>36</v>
       </c>
       <c r="C23">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="D23">
         <f t="shared" si="0"/>
-        <v>24.75</v>
+        <v>55</v>
       </c>
       <c r="E23">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="F23">
-        <v>100</v>
+        <v>260</v>
       </c>
       <c r="G23">
         <v>1</v>
+      </c>
+      <c r="H23" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1301,6 +1343,9 @@
       <c r="G25">
         <v>1</v>
       </c>
+      <c r="H25" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
@@ -1349,6 +1394,9 @@
       <c r="G27">
         <v>1</v>
       </c>
+      <c r="H27" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
@@ -1373,6 +1421,9 @@
       <c r="G28">
         <v>1</v>
       </c>
+      <c r="H28" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
@@ -1397,6 +1448,9 @@
       <c r="G29">
         <v>1</v>
       </c>
+      <c r="H29" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
@@ -1499,6 +1553,9 @@
       <c r="G33">
         <v>1</v>
       </c>
+      <c r="H33" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
@@ -1655,6 +1712,9 @@
       <c r="G39">
         <v>1</v>
       </c>
+      <c r="H39" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
@@ -1679,6 +1739,9 @@
       <c r="G40">
         <v>1</v>
       </c>
+      <c r="H40" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
@@ -1715,20 +1778,23 @@
         <v>53</v>
       </c>
       <c r="C42">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="D42">
         <f t="shared" si="0"/>
-        <v>2.25</v>
+        <v>122.5</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F42">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="G42">
         <v>1</v>
+      </c>
+      <c r="H42" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -1805,6 +1871,9 @@
       <c r="G45">
         <v>2</v>
       </c>
+      <c r="H45" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
@@ -1883,6 +1952,9 @@
       <c r="G48">
         <v>1</v>
       </c>
+      <c r="H48" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49">
@@ -1907,6 +1979,9 @@
       <c r="G49">
         <v>1</v>
       </c>
+      <c r="H49" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50">
@@ -1931,6 +2006,9 @@
       <c r="G50">
         <v>1</v>
       </c>
+      <c r="H50" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51">
@@ -1955,6 +2033,9 @@
       <c r="G51">
         <v>1</v>
       </c>
+      <c r="H51" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52">
@@ -1979,6 +2060,9 @@
       <c r="G52">
         <v>1</v>
       </c>
+      <c r="H52" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53">
@@ -2002,6 +2086,9 @@
       </c>
       <c r="G53">
         <v>1</v>
+      </c>
+      <c r="H53" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>